<commit_message>
Add data validation and dropdown lists to Excel templates; refactor VentasImportController error handling
</commit_message>
<xml_diff>
--- a/Backend/public/docs/ventas-consumidor-final-format.xlsx
+++ b/Backend/public/docs/ventas-consumidor-final-format.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="54">
   <si>
     <t>nombre</t>
   </si>
@@ -126,12 +126,18 @@
     <t>- Las filas se agruparán en ventas según el cliente y la fecha.</t>
   </si>
   <si>
+    <t>- Utilice las listas desplegables para seleccionar valores en tipo de documento, tipo de ítem, forma de pago y condición.</t>
+  </si>
+  <si>
     <t>2. CAMPOS OBLIGATORIOS:</t>
   </si>
   <si>
     <t>- nombre: Nombre del cliente (o "Consumidor Final").</t>
   </si>
   <si>
+    <t>- tipo_documento: Seleccione de la lista desplegable (DUI, NIT, Pasaporte, etc.)</t>
+  </si>
+  <si>
     <t>- fecha: Fecha de la venta en formato YYYY-MM-DD.</t>
   </si>
   <si>
@@ -162,7 +168,7 @@
     <t>5. FORMAS DE PAGO:</t>
   </si>
   <si>
-    <t>- Efectivo, Tarjeta, Cheque, Transferencia, Crédito, etc.</t>
+    <t>- Efectivo, Tarjeta de crédito/débito, Cheque, Transferencia, CARGO AUTOMATICO.</t>
   </si>
   <si>
     <t>6. CONDICIÓN:</t>
@@ -691,6 +697,32 @@
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
+  <dataValidations count="8">
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="B2:B101">
+      <formula1>"DUI,NIT,Pasaporte,Carnet de residente,Otro"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="K2:K101">
+      <formula1>"Producto,Servicio"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="L2:L101">
+      <formula1>"Efectivo,Tarjeta de crédito/débito,Cheque,Transferencia,CARGO AUTOMATICO"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="S2:S101">
+      <formula1>"Contado,Crédito"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="B2">
+      <formula1>"DUI,NIT,Pasaporte,Carnet de residente,Otro"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="K2">
+      <formula1>"Producto,Servicio"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="L2">
+      <formula1>"Efectivo,Tarjeta de crédito/débito,Cheque,Transferencia,CARGO AUTOMATICO"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="S2">
+      <formula1>"Contado,Crédito"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
@@ -711,7 +743,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="true" style="0"/>
@@ -743,13 +775,13 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="1" t="s">
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>37</v>
       </c>
     </row>
@@ -768,59 +800,69 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="1" t="s">
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
         <v>41</v>
       </c>
     </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>42</v>
+      </c>
+    </row>
     <row r="17" spans="1:2">
-      <c r="A17" t="s">
-        <v>42</v>
+      <c r="A17" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="1" t="s">
         <v>44</v>
       </c>
     </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>45</v>
+      <c r="A21" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="1" t="s">
         <v>47</v>
       </c>
     </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>48</v>
+      </c>
+    </row>
     <row r="25" spans="1:2">
-      <c r="A25" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="A27" s="1" t="s">
+      <c r="A25" s="1" t="s">
         <v>49</v>
       </c>
     </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+    </row>
     <row r="28" spans="1:2">
-      <c r="A28" t="s">
-        <v>50</v>
+      <c r="A28" s="1" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor GenerarPlantillasCommand; remove example data and simplify dropdown options for improved clarity
</commit_message>
<xml_diff>
--- a/Backend/public/docs/ventas-consumidor-final-format.xlsx
+++ b/Backend/public/docs/ventas-consumidor-final-format.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="43">
   <si>
     <t>nombre</t>
   </si>
@@ -76,39 +76,6 @@
   </si>
   <si>
     <t>fecha_pago</t>
-  </si>
-  <si>
-    <t>Juan Pérez</t>
-  </si>
-  <si>
-    <t>DUI</t>
-  </si>
-  <si>
-    <t>01234567-8</t>
-  </si>
-  <si>
-    <t>Residencial Las Flores, Casa #10</t>
-  </si>
-  <si>
-    <t>7777-8888</t>
-  </si>
-  <si>
-    <t>juan.perez@email.com</t>
-  </si>
-  <si>
-    <t>2025-03-25</t>
-  </si>
-  <si>
-    <t>Reparación de laptop</t>
-  </si>
-  <si>
-    <t>Servicio</t>
-  </si>
-  <si>
-    <t>Tarjeta de crédito/débito</t>
-  </si>
-  <si>
-    <t>Contado</t>
   </si>
   <si>
     <t>INSTRUCCIONES PARA IMPORTAR VENTAS (CONSUMIDOR FINAL)</t>
@@ -549,18 +516,18 @@
   <dimension ref="A1:T2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="8" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="17" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="16" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="19" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="16" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="38" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="11" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="24" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="12" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="24" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="11" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="10" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="8" bestFit="true" customWidth="true" style="0"/>
+    <col min="9" max="9" width="6" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="13" bestFit="true" customWidth="true" style="0"/>
     <col min="11" max="11" width="11" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="30" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="12" bestFit="true" customWidth="true" style="0"/>
     <col min="13" max="13" width="8" bestFit="true" customWidth="true" style="0"/>
     <col min="14" max="14" width="9" bestFit="true" customWidth="true" style="0"/>
     <col min="15" max="15" width="10" bestFit="true" customWidth="true" style="0"/>
@@ -634,66 +601,10 @@
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>50.0</v>
-      </c>
-      <c r="O2">
-        <v>50.0</v>
-      </c>
-      <c r="P2">
-        <v>6.5</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2">
-        <v>56.5</v>
-      </c>
-      <c r="S2" t="s">
-        <v>30</v>
-      </c>
-      <c r="T2" t="s">
-        <v>26</v>
-      </c>
+      <c r="B2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="S2"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
@@ -702,10 +613,10 @@
       <formula1>"DUI,NIT,Pasaporte,Carnet de residente,Otro"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="K2:K101">
-      <formula1>"Producto,Servicio"</formula1>
+      <formula1>"Servicio"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="L2:L101">
-      <formula1>"Efectivo,Tarjeta de crédito/débito,Cheque,Transferencia,CARGO AUTOMATICO"</formula1>
+      <formula1>"Tarjeta de crédito/débito"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="S2:S101">
       <formula1>"Contado,Crédito"</formula1>
@@ -714,10 +625,10 @@
       <formula1>"DUI,NIT,Pasaporte,Carnet de residente,Otro"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="K2">
-      <formula1>"Producto,Servicio"</formula1>
+      <formula1>"Servicio"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="L2">
-      <formula1>"Efectivo,Tarjeta de crédito/débito,Cheque,Transferencia,CARGO AUTOMATICO"</formula1>
+      <formula1>"Tarjeta de crédito/débito"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="information" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="S2">
       <formula1>"Contado,Crédito"</formula1>
@@ -752,117 +663,117 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="1" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor GenerarPlantillasCommand; update department and municipality codes for accuracy, and simplify payment methods for clarity
</commit_message>
<xml_diff>
--- a/Backend/public/docs/ventas-consumidor-final-format.xlsx
+++ b/Backend/public/docs/ventas-consumidor-final-format.xlsx
@@ -117,10 +117,10 @@
     <t>3. CÓDIGOS DE DEPARTAMENTOS Y MUNICIPIOS:</t>
   </si>
   <si>
-    <t>- Los códigos de departamento deben corresponder a los registrados en el sistema (ej. 01 para San Salvador).</t>
-  </si>
-  <si>
-    <t>- Los códigos de municipio deben corresponder a los registrados en el sistema (ej. 0101 para San Salvador).</t>
+    <t>- Los códigos de departamento deben corresponder a los registrados en el sistema (ej. 6 para San Salvador).</t>
+  </si>
+  <si>
+    <t>- Los códigos de municipio deben corresponder a los registrados en el sistema (ej. 24 para San Salvador).</t>
   </si>
   <si>
     <t>4. TIPOS DE ÍTEM:</t>
@@ -135,7 +135,7 @@
     <t>5. FORMAS DE PAGO:</t>
   </si>
   <si>
-    <t>- Efectivo, Tarjeta de crédito/débito, Cheque, Transferencia, CARGO AUTOMATICO.</t>
+    <t>- Efectivo, Tarjeta de crédito/débito</t>
   </si>
   <si>
     <t>6. CONDICIÓN:</t>

</xml_diff>